<commit_message>
Add resume outreach workflow and agency tracker assets
</commit_message>
<xml_diff>
--- a/resumes/uae-job-opening-scan.xlsx
+++ b/resumes/uae-job-opening-scan.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M102"/>
+  <dimension ref="A1:M103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2230,12 +2230,24 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>To Contact</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr"/>
-      <c r="F37" s="2" t="inlineStr"/>
-      <c r="G37" s="2" t="inlineStr"/>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>ATS 86/100. Tailored resume: resumes/property-finder-product-designer-resume.md. Report: resumes/property-finder-product-designer-ats-report.md. Figma: https://www.figma.com/design/or9EJUqIuF1yN5SEJ15LtP | Gmail sent id: 19e896596bf0a734</t>
+        </is>
+      </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
           <t>Opening Found</t>
@@ -2258,7 +2270,7 @@
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>Tailor resume and apply</t>
+          <t>Apply now with tailored resume and email</t>
         </is>
       </c>
       <c r="M37" s="2" t="inlineStr">
@@ -2669,12 +2681,24 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>To Contact</t>
-        </is>
-      </c>
-      <c r="E46" s="3" t="inlineStr"/>
-      <c r="F46" s="3" t="inlineStr"/>
-      <c r="G46" s="3" t="inlineStr"/>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>Agency outreach sent with UAE Product Designer CV. Gmail sent id: 19e89945308caee8</t>
+        </is>
+      </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
           <t>Needs Manual Check</t>
@@ -2689,7 +2713,7 @@
       </c>
       <c r="L46" s="3" t="inlineStr">
         <is>
-          <t>Run company careers/LinkedIn check</t>
+          <t>Follow up if no response</t>
         </is>
       </c>
       <c r="M46" s="3" t="inlineStr">
@@ -2716,12 +2740,24 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>To Contact</t>
-        </is>
-      </c>
-      <c r="E47" s="3" t="inlineStr"/>
-      <c r="F47" s="3" t="inlineStr"/>
-      <c r="G47" s="3" t="inlineStr"/>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>Agency outreach sent with UAE Product Designer CV. Gmail sent id: 19e899494cedcd60</t>
+        </is>
+      </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
           <t>Needs Manual Check</t>
@@ -2736,7 +2772,7 @@
       </c>
       <c r="L47" s="3" t="inlineStr">
         <is>
-          <t>Run company careers/LinkedIn check</t>
+          <t>Follow up if no response</t>
         </is>
       </c>
       <c r="M47" s="3" t="inlineStr">
@@ -2763,12 +2799,24 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>To Contact</t>
-        </is>
-      </c>
-      <c r="E48" s="3" t="inlineStr"/>
-      <c r="F48" s="3" t="inlineStr"/>
-      <c r="G48" s="3" t="inlineStr"/>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>Agency outreach sent with UAE Product Designer CV. Gmail sent id: 19e8994d82744ae3</t>
+        </is>
+      </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
           <t>Needs Manual Check</t>
@@ -2783,7 +2831,7 @@
       </c>
       <c r="L48" s="3" t="inlineStr">
         <is>
-          <t>Run company careers/LinkedIn check</t>
+          <t>Follow up if no response</t>
         </is>
       </c>
       <c r="M48" s="3" t="inlineStr">
@@ -2810,12 +2858,24 @@
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>To Contact</t>
-        </is>
-      </c>
-      <c r="E49" s="3" t="inlineStr"/>
-      <c r="F49" s="3" t="inlineStr"/>
-      <c r="G49" s="3" t="inlineStr"/>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>Agency outreach sent with UAE Product Designer CV. Gmail sent id: 19e89951d50b68b7</t>
+        </is>
+      </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
           <t>Needs Manual Check</t>
@@ -2830,7 +2890,7 @@
       </c>
       <c r="L49" s="3" t="inlineStr">
         <is>
-          <t>Run company careers/LinkedIn check</t>
+          <t>Follow up if no response</t>
         </is>
       </c>
       <c r="M49" s="3" t="inlineStr">
@@ -2857,12 +2917,24 @@
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>To Contact</t>
-        </is>
-      </c>
-      <c r="E50" s="3" t="inlineStr"/>
-      <c r="F50" s="3" t="inlineStr"/>
-      <c r="G50" s="3" t="inlineStr"/>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>Agency outreach sent with UAE Product Designer CV. Gmail sent id: 19e89956b48c3cad</t>
+        </is>
+      </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
           <t>Needs Manual Check</t>
@@ -2877,7 +2949,7 @@
       </c>
       <c r="L50" s="3" t="inlineStr">
         <is>
-          <t>Run company careers/LinkedIn check</t>
+          <t>Follow up if no response</t>
         </is>
       </c>
       <c r="M50" s="3" t="inlineStr">
@@ -2904,12 +2976,24 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>To Contact</t>
-        </is>
-      </c>
-      <c r="E51" s="3" t="inlineStr"/>
-      <c r="F51" s="3" t="inlineStr"/>
-      <c r="G51" s="3" t="inlineStr"/>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>Agency outreach sent with UAE Product Designer CV. Gmail sent id: 19e8995bb9aefbbb</t>
+        </is>
+      </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
           <t>Needs Manual Check</t>
@@ -2924,7 +3008,7 @@
       </c>
       <c r="L51" s="3" t="inlineStr">
         <is>
-          <t>Run company careers/LinkedIn check</t>
+          <t>Follow up if no response</t>
         </is>
       </c>
       <c r="M51" s="3" t="inlineStr">
@@ -2951,12 +3035,24 @@
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>To Contact</t>
-        </is>
-      </c>
-      <c r="E52" s="3" t="inlineStr"/>
-      <c r="F52" s="3" t="inlineStr"/>
-      <c r="G52" s="3" t="inlineStr"/>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>Agency outreach sent with UAE Product Designer CV. Gmail sent id: 19e8995fe4f14b21</t>
+        </is>
+      </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
           <t>Needs Manual Check</t>
@@ -2971,7 +3067,7 @@
       </c>
       <c r="L52" s="3" t="inlineStr">
         <is>
-          <t>Run company careers/LinkedIn check</t>
+          <t>Follow up if no response</t>
         </is>
       </c>
       <c r="M52" s="3" t="inlineStr">
@@ -2998,12 +3094,24 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>To Contact</t>
-        </is>
-      </c>
-      <c r="E53" s="3" t="inlineStr"/>
-      <c r="F53" s="3" t="inlineStr"/>
-      <c r="G53" s="3" t="inlineStr"/>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>Agency outreach sent with UAE Product Designer CV. Gmail sent id: 19e8996472185e94</t>
+        </is>
+      </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
           <t>Needs Manual Check</t>
@@ -3018,7 +3126,7 @@
       </c>
       <c r="L53" s="3" t="inlineStr">
         <is>
-          <t>Run company careers/LinkedIn check</t>
+          <t>Follow up if no response</t>
         </is>
       </c>
       <c r="M53" s="3" t="inlineStr">
@@ -3045,12 +3153,24 @@
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>To Contact</t>
-        </is>
-      </c>
-      <c r="E54" s="3" t="inlineStr"/>
-      <c r="F54" s="3" t="inlineStr"/>
-      <c r="G54" s="3" t="inlineStr"/>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>Agency outreach sent with UAE Product Designer CV. Gmail sent id: 19e8996a624036db</t>
+        </is>
+      </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
           <t>Needs Manual Check</t>
@@ -3065,7 +3185,7 @@
       </c>
       <c r="L54" s="3" t="inlineStr">
         <is>
-          <t>Run company careers/LinkedIn check</t>
+          <t>Follow up if no response</t>
         </is>
       </c>
       <c r="M54" s="3" t="inlineStr">
@@ -3092,12 +3212,24 @@
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>To Contact</t>
-        </is>
-      </c>
-      <c r="E55" s="3" t="inlineStr"/>
-      <c r="F55" s="3" t="inlineStr"/>
-      <c r="G55" s="3" t="inlineStr"/>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>BAC-specific CV sent. Gmail sent id: 19e89c01053d2189</t>
+        </is>
+      </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
           <t>Needs Manual Check</t>
@@ -3112,7 +3244,7 @@
       </c>
       <c r="L55" s="3" t="inlineStr">
         <is>
-          <t>Run company careers/LinkedIn check</t>
+          <t>Follow up if no response</t>
         </is>
       </c>
       <c r="M55" s="3" t="inlineStr">
@@ -5325,6 +5457,73 @@
         </is>
       </c>
       <c r="M102" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Ziina</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>anton.badashov@ziina.com; jocelyn.meyer@ziina.com</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Direct Employer</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Sent tailored Ziina fintech CV. Gmail sent id: 19e898b575624043</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Opening Found</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>Senior Product Designer</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/ziina/jobs/4631469101</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>Follow up in one week if no reply</t>
+        </is>
+      </c>
+      <c r="M103" t="inlineStr">
         <is>
           <t>2026-06-02</t>
         </is>

</xml_diff>

<commit_message>
Recover job-hunt context and tailor Amwal resume
</commit_message>
<xml_diff>
--- a/resumes/uae-job-opening-scan.xlsx
+++ b/resumes/uae-job-opening-scan.xlsx
@@ -2696,7 +2696,7 @@
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>Agency outreach sent with UAE Product Designer CV. Gmail sent id: 19e89945308caee8</t>
+          <t>Agency outreach sent with UAE Product Designer CV. Gmail sent id: 19e89945308caee8 | Duplicate resend approved by user; Gmail sent id: 19e89cf5ce9cc34b</t>
         </is>
       </c>
       <c r="H46" s="3" t="inlineStr">
@@ -2755,7 +2755,7 @@
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>Agency outreach sent with UAE Product Designer CV. Gmail sent id: 19e899494cedcd60</t>
+          <t>Agency outreach sent with UAE Product Designer CV. Gmail sent id: 19e899494cedcd60 | Duplicate resend approved by user; Gmail sent id: 19e89cfc2a56acd0</t>
         </is>
       </c>
       <c r="H47" s="3" t="inlineStr">
@@ -2814,7 +2814,7 @@
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>Agency outreach sent with UAE Product Designer CV. Gmail sent id: 19e8994d82744ae3</t>
+          <t>Agency outreach sent with UAE Product Designer CV. Gmail sent id: 19e8994d82744ae3 | Duplicate resend approved by user; Gmail sent id: 19e89d0228492b70</t>
         </is>
       </c>
       <c r="H48" s="3" t="inlineStr">
@@ -2873,7 +2873,7 @@
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>Agency outreach sent with UAE Product Designer CV. Gmail sent id: 19e89951d50b68b7</t>
+          <t>Agency outreach sent with UAE Product Designer CV. Gmail sent id: 19e89951d50b68b7 | Duplicate resend approved by user; Gmail sent id: 19e89d089904515a</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr">
@@ -2932,7 +2932,7 @@
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>Agency outreach sent with UAE Product Designer CV. Gmail sent id: 19e89956b48c3cad</t>
+          <t>Agency outreach sent with UAE Product Designer CV. Gmail sent id: 19e89956b48c3cad | Duplicate resend approved by user; Gmail sent id: 19e89d0ead50a17f</t>
         </is>
       </c>
       <c r="H50" s="3" t="inlineStr">
@@ -2991,7 +2991,7 @@
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>Agency outreach sent with UAE Product Designer CV. Gmail sent id: 19e8995bb9aefbbb</t>
+          <t>Agency outreach sent with UAE Product Designer CV. Gmail sent id: 19e8995bb9aefbbb | Duplicate resend approved by user; Gmail sent id: 19e89d146678c6a2</t>
         </is>
       </c>
       <c r="H51" s="3" t="inlineStr">
@@ -3050,7 +3050,7 @@
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>Agency outreach sent with UAE Product Designer CV. Gmail sent id: 19e8995fe4f14b21</t>
+          <t>Agency outreach sent with UAE Product Designer CV. Gmail sent id: 19e8995fe4f14b21 | Duplicate resend approved by user; Gmail sent id: 19e89d1b128adb5c</t>
         </is>
       </c>
       <c r="H52" s="3" t="inlineStr">
@@ -3109,7 +3109,7 @@
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>Agency outreach sent with UAE Product Designer CV. Gmail sent id: 19e8996472185e94</t>
+          <t>Agency outreach sent with UAE Product Designer CV. Gmail sent id: 19e8996472185e94 | Duplicate resend approved by user; Gmail sent id: 19e89d20d8adcac1</t>
         </is>
       </c>
       <c r="H53" s="3" t="inlineStr">
@@ -3168,7 +3168,7 @@
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t>Agency outreach sent with UAE Product Designer CV. Gmail sent id: 19e8996a624036db</t>
+          <t>Agency outreach sent with UAE Product Designer CV. Gmail sent id: 19e8996a624036db | Duplicate resend approved by user; Gmail sent id: 19e89d28a4d760b1</t>
         </is>
       </c>
       <c r="H54" s="3" t="inlineStr">

</xml_diff>